<commit_message>
Use real Lucobond stock sizes and add cutting layout diagrams
Update stock plates to the in-stock sizes (1000x2000, 1000x3000,
1220x2440, 1500x3000) and regenerate the cut plan (now 12% waste). Add
render_layout.py producing a per-plate cutting diagram PDF, grouping
identical layouts.

https://claude.ai/code/session_01KNfHFGm3BZAV2u3TfGKXLF
</commit_message>
<xml_diff>
--- a/sheet_metal_calc.xlsx
+++ b/sheet_metal_calc.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="סיכום" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="רשימת פאנלים" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="פירוט 1500x3000" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="פירוט 1000x3000" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -543,89 +543,105 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>1250x2500</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>101</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>315.62</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>0.2835</v>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>1000x3000</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>258</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.1234</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>1220x2440</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>117</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>348.29</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0.3507</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>1500x3000</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B6" s="3" t="n">
         <v>64</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C6" s="3" t="n">
         <v>288</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D6" s="4" t="n">
         <v>0.2147</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>שטח נדרש נטו (מ"ר):</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B8" s="8" t="n">
         <v>226.16</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>המלצה:</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>1500x3000 → 64 לוחות, פחת 21%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>הנחות:</t>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>1000x3000 → 86 לוחות, פחת 12%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>• תפרים מותרים (פאנל מורכב מכמה לוחות).</t>
+          <t>הנחות:</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>• ללא חפיפות וללא קרף חיתוך.</t>
+          <t>• תפרים מותרים (פאנל מורכב מכמה לוחות).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>• ניצול שאריות בין פאנלים.</t>
+          <t>• ללא חפיפות וללא קרף חיתוך.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>• ניצול שאריות בין פאנלים.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>• סיבוב חתיכות חופשי (אם לפח יש כיוון - יש לחשב מחדש).</t>
         </is>
@@ -930,7 +946,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>פירוט לפי סוג פאנל - לוח 1500x3000</t>
+          <t>פירוט לפי סוג פאנל - לוח 1000x3000</t>
         </is>
       </c>
     </row>
@@ -966,10 +982,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -982,10 +998,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -998,10 +1014,10 @@
         <v>6</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -1081,7 +1097,7 @@
         <v>2</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
@@ -1097,20 +1113,20 @@
         <v>1</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>סכום עצמאי: 76 לוחות</t>
+          <t>סכום עצמאי: 96 לוחות</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>בפועל עם ניצול שאריות משותף: 64 לוחות (פחות מהסכום העצמאי).</t>
+          <t>בפועל עם ניצול שאריות משותף: 86 לוחות (פחות מהסכום העצמאי).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add panel pricing (material cost + 30%) and switch to cost-optimal nesting
Add plate purchase prices, optimize plate choice by cost instead of area,
and add build_pricing.py producing a per-panel quote (unit price incl.
30% markup) plus totals and real margin after shared nesting.

https://claude.ai/code/session_01KNfHFGm3BZAV2u3TfGKXLF
</commit_message>
<xml_diff>
--- a/sheet_metal_calc.xlsx
+++ b/sheet_metal_calc.xlsx
@@ -561,17 +561,17 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>1220x2440</t>
+          <t>1250x2500</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>348.29</v>
+        <v>315.62</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.3507</v>
+        <v>0.2835</v>
       </c>
     </row>
     <row r="6">

</xml_diff>